<commit_message>
Continuando dia 04.03.2026 -> Início da prototipagem no Figma, link do README.
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zdusa\OneDrive\Documentos\ZDU\Criacao de Jogos\Games\Clicker-Lizard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{429CC2C4-3FF2-4623-AF65-A91EFF516DBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D12CBAA1-60A8-444F-949B-1A39A56053D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="147">
   <si>
     <t>PRODUCT BACKLOG - ZENLYX</t>
   </si>
@@ -729,6 +729,18 @@
   </si>
   <si>
     <t>Motivo para Jogar</t>
+  </si>
+  <si>
+    <t>Requisito Dividido</t>
+  </si>
+  <si>
+    <t>Parte do Requisito</t>
+  </si>
+  <si>
+    <t>Layout</t>
+  </si>
+  <si>
+    <t>Tela Inicial</t>
   </si>
 </sst>
 </file>
@@ -970,14 +982,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1109,6 +1115,13 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2593,1076 +2606,1076 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="I1" s="2" t="s">
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="I1" s="63" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
     </row>
     <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="4"/>
-      <c r="J2" s="5" t="s">
+      <c r="I2" s="2"/>
+      <c r="J2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="K2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="L2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="M2" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6"/>
-      <c r="B3" s="7" t="s">
+      <c r="A3" s="4"/>
+      <c r="B3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="9"/>
-      <c r="I3" s="10" t="s">
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="7"/>
+      <c r="I3" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="J3" s="11">
+      <c r="J3" s="9">
         <f>SUM(E4:E5,E7:E17,E19:E25,E27:E38,E40:E44)</f>
         <v>328</v>
       </c>
-      <c r="K3" s="11">
+      <c r="K3" s="9">
         <f>SUM(K4:K8)</f>
         <v>207</v>
       </c>
-      <c r="L3" s="11">
+      <c r="L3" s="9">
         <f>J3</f>
         <v>328</v>
       </c>
-      <c r="M3" s="11">
+      <c r="M3" s="9">
         <f>J3</f>
         <v>328</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="15">
+      <c r="E4" s="13">
         <v>5</v>
       </c>
-      <c r="F4" s="15">
+      <c r="F4" s="13">
         <v>2</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="J4" s="11">
+      <c r="J4" s="9">
         <f>SUM(E4:E5)</f>
         <v>13</v>
       </c>
-      <c r="K4" s="11">
+      <c r="K4" s="9">
         <f>E4+E5</f>
         <v>13</v>
       </c>
-      <c r="L4" s="11">
+      <c r="L4" s="9">
         <f t="shared" ref="L4:M6" si="0">L3-J4</f>
         <v>315</v>
       </c>
-      <c r="M4" s="11">
+      <c r="M4" s="9">
         <f t="shared" si="0"/>
         <v>315</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E5" s="15">
+      <c r="E5" s="13">
         <v>8</v>
       </c>
-      <c r="F5" s="15">
+      <c r="F5" s="13">
         <v>1</v>
       </c>
-      <c r="G5" s="15" t="s">
+      <c r="G5" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="J5" s="11">
+      <c r="J5" s="9">
         <f>SUM(E7:E17)</f>
         <v>102</v>
       </c>
-      <c r="K5" s="11">
+      <c r="K5" s="9">
         <f>E7+E8+E9</f>
         <v>31</v>
       </c>
-      <c r="L5" s="11">
+      <c r="L5" s="9">
         <f t="shared" si="0"/>
         <v>213</v>
       </c>
-      <c r="M5" s="11">
+      <c r="M5" s="9">
         <f t="shared" si="0"/>
         <v>284</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="17"/>
-      <c r="B6" s="18" t="s">
+      <c r="A6" s="15"/>
+      <c r="B6" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="19"/>
-      <c r="I6" s="4" t="s">
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="17"/>
+      <c r="I6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="J6" s="11">
+      <c r="J6" s="9">
         <f>SUM(E19:E25)</f>
         <v>55</v>
       </c>
-      <c r="K6" s="11">
+      <c r="K6" s="9">
         <f>E11+E12+E13+E15+E14+E16+E17+E19+E20</f>
         <v>74</v>
       </c>
-      <c r="L6" s="11">
+      <c r="L6" s="9">
         <f t="shared" si="0"/>
         <v>158</v>
       </c>
-      <c r="M6" s="11">
+      <c r="M6" s="9">
         <f t="shared" si="0"/>
         <v>210</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="22" t="s">
+      <c r="C7" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="23" t="s">
+      <c r="D7" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="23">
+      <c r="E7" s="21">
         <v>21</v>
       </c>
-      <c r="F7" s="23">
+      <c r="F7" s="21">
         <v>1</v>
       </c>
-      <c r="G7" s="23" t="s">
+      <c r="G7" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J7" s="11">
+      <c r="J7" s="9">
         <f>SUM(E27:E38)</f>
         <v>121</v>
       </c>
-      <c r="K7" s="11">
+      <c r="K7" s="9">
         <f>E21+E23+E24+E25+E27+E28+E29+E34+E36</f>
         <v>76</v>
       </c>
-      <c r="L7" s="11">
+      <c r="L7" s="9">
         <f>L6-J7</f>
         <v>37</v>
       </c>
-      <c r="M7" s="11">
+      <c r="M7" s="9">
         <f>M6-K7</f>
         <v>134</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="20" t="s">
+      <c r="A8" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="C8" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="23" t="s">
+      <c r="D8" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="23">
+      <c r="E8" s="21">
         <v>5</v>
       </c>
-      <c r="F8" s="23">
+      <c r="F8" s="21">
         <v>10</v>
       </c>
-      <c r="G8" s="23" t="s">
+      <c r="G8" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="I8" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="J8" s="11">
+      <c r="J8" s="9">
         <f>SUM(E40:E44)</f>
         <v>37</v>
       </c>
-      <c r="K8" s="11">
+      <c r="K8" s="9">
         <f>E35+E37</f>
         <v>13</v>
       </c>
-      <c r="L8" s="11">
+      <c r="L8" s="9">
         <f>L7-J8</f>
         <v>0</v>
       </c>
-      <c r="M8" s="11">
+      <c r="M8" s="9">
         <f>M7-K8</f>
         <v>121</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="25" t="s">
+      <c r="A9" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="C9" s="22" t="s">
+      <c r="C9" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="23" t="s">
+      <c r="D9" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="23">
+      <c r="E9" s="21">
         <v>5</v>
       </c>
-      <c r="F9" s="23">
+      <c r="F9" s="21">
         <v>9</v>
       </c>
-      <c r="G9" s="23" t="s">
+      <c r="G9" s="21" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="25" t="s">
+      <c r="A10" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="22" t="s">
+      <c r="C10" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="23" t="s">
+      <c r="D10" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="E10" s="23">
+      <c r="E10" s="21">
         <v>13</v>
       </c>
-      <c r="F10" s="23">
+      <c r="F10" s="21">
         <v>2</v>
       </c>
-      <c r="G10" s="23" t="s">
+      <c r="G10" s="21" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="25" t="s">
+      <c r="A11" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="26" t="s">
+      <c r="B11" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="22" t="s">
+      <c r="C11" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="23" t="s">
+      <c r="D11" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="E11" s="23">
+      <c r="E11" s="21">
         <v>3</v>
       </c>
-      <c r="F11" s="23">
+      <c r="F11" s="21">
         <v>11</v>
       </c>
-      <c r="G11" s="23" t="s">
+      <c r="G11" s="21" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="27" t="s">
+      <c r="A12" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="C12" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="23" t="s">
+      <c r="D12" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="23">
+      <c r="E12" s="21">
         <v>8</v>
       </c>
-      <c r="F12" s="23">
+      <c r="F12" s="21">
         <v>3</v>
       </c>
-      <c r="G12" s="23" t="s">
+      <c r="G12" s="21" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="27" t="s">
+      <c r="A13" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="B13" s="24" t="s">
+      <c r="B13" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="22" t="s">
+      <c r="C13" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="D13" s="23" t="s">
+      <c r="D13" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="E13" s="23">
+      <c r="E13" s="21">
         <v>5</v>
       </c>
-      <c r="F13" s="23">
+      <c r="F13" s="21">
         <v>4</v>
       </c>
-      <c r="G13" s="23" t="s">
+      <c r="G13" s="21" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="27" t="s">
+      <c r="A14" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="B14" s="24" t="s">
+      <c r="B14" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="22" t="s">
+      <c r="C14" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="D14" s="23" t="s">
+      <c r="D14" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="E14" s="23">
+      <c r="E14" s="21">
         <v>5</v>
       </c>
-      <c r="F14" s="23">
+      <c r="F14" s="21">
         <v>5</v>
       </c>
-      <c r="G14" s="23" t="s">
+      <c r="G14" s="21" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="27" t="s">
+      <c r="A15" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="B15" s="24" t="s">
+      <c r="B15" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="C15" s="22" t="s">
+      <c r="C15" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="D15" s="23" t="s">
+      <c r="D15" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="E15" s="23">
+      <c r="E15" s="21">
         <v>8</v>
       </c>
-      <c r="F15" s="23">
+      <c r="F15" s="21">
         <v>8</v>
       </c>
-      <c r="G15" s="23" t="s">
+      <c r="G15" s="21" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="27" t="s">
+      <c r="A16" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="B16" s="24" t="s">
+      <c r="B16" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="C16" s="22" t="s">
+      <c r="C16" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="D16" s="23" t="s">
+      <c r="D16" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="E16" s="23">
+      <c r="E16" s="21">
         <v>8</v>
       </c>
-      <c r="F16" s="23">
+      <c r="F16" s="21">
         <v>7</v>
       </c>
-      <c r="G16" s="23" t="s">
+      <c r="G16" s="21" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="25" t="s">
+      <c r="A17" s="23" t="s">
         <v>50</v>
       </c>
-      <c r="B17" s="28" t="s">
+      <c r="B17" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="C17" s="22" t="s">
+      <c r="C17" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="D17" s="23" t="s">
+      <c r="D17" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="E17" s="23">
+      <c r="E17" s="21">
         <v>21</v>
       </c>
-      <c r="F17" s="23">
+      <c r="F17" s="21">
         <v>6</v>
       </c>
-      <c r="G17" s="23" t="s">
+      <c r="G17" s="21" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="29"/>
-      <c r="B18" s="30" t="s">
+      <c r="A18" s="27"/>
+      <c r="B18" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="31"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="31"/>
-      <c r="F18" s="31"/>
-      <c r="G18" s="32"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="29"/>
+      <c r="G18" s="30"/>
     </row>
     <row r="19" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="33" t="s">
+      <c r="A19" s="31" t="s">
         <v>52</v>
       </c>
-      <c r="B19" s="34" t="s">
+      <c r="B19" s="32" t="s">
         <v>53</v>
       </c>
-      <c r="C19" s="35" t="s">
+      <c r="C19" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="36" t="s">
+      <c r="D19" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="E19" s="36">
+      <c r="E19" s="34">
         <v>8</v>
       </c>
-      <c r="F19" s="36">
+      <c r="F19" s="34">
         <v>1</v>
       </c>
-      <c r="G19" s="36" t="s">
+      <c r="G19" s="34" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="33" t="s">
+      <c r="A20" s="31" t="s">
         <v>54</v>
       </c>
-      <c r="B20" s="37" t="s">
+      <c r="B20" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="35" t="s">
+      <c r="C20" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="D20" s="36" t="s">
+      <c r="D20" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="E20" s="36">
+      <c r="E20" s="34">
         <v>8</v>
       </c>
-      <c r="F20" s="36">
+      <c r="F20" s="34">
         <v>2</v>
       </c>
-      <c r="G20" s="36" t="s">
+      <c r="G20" s="34" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="38" t="s">
+      <c r="A21" s="36" t="s">
         <v>56</v>
       </c>
-      <c r="B21" s="39" t="s">
+      <c r="B21" s="37" t="s">
         <v>57</v>
       </c>
-      <c r="C21" s="35" t="s">
+      <c r="C21" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="D21" s="36" t="s">
+      <c r="D21" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="E21" s="36">
+      <c r="E21" s="34">
         <v>8</v>
       </c>
-      <c r="F21" s="36">
+      <c r="F21" s="34">
         <v>3</v>
       </c>
-      <c r="G21" s="36" t="s">
+      <c r="G21" s="34" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="33" t="s">
+      <c r="A22" s="31" t="s">
         <v>58</v>
       </c>
-      <c r="B22" s="40" t="s">
+      <c r="B22" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="C22" s="35" t="s">
+      <c r="C22" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="D22" s="36" t="s">
+      <c r="D22" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="E22" s="36">
+      <c r="E22" s="34">
         <v>5</v>
       </c>
-      <c r="F22" s="36">
+      <c r="F22" s="34">
         <v>4</v>
       </c>
-      <c r="G22" s="36" t="s">
+      <c r="G22" s="34" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="33" t="s">
+      <c r="A23" s="31" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="40" t="s">
+      <c r="B23" s="38" t="s">
         <v>61</v>
       </c>
-      <c r="C23" s="35" t="s">
+      <c r="C23" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="D23" s="36" t="s">
+      <c r="D23" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="E23" s="36">
+      <c r="E23" s="34">
         <v>5</v>
       </c>
-      <c r="F23" s="36">
+      <c r="F23" s="34">
         <v>5</v>
       </c>
-      <c r="G23" s="36" t="s">
+      <c r="G23" s="34" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="33" t="s">
+      <c r="A24" s="31" t="s">
         <v>62</v>
       </c>
-      <c r="B24" s="40" t="s">
+      <c r="B24" s="38" t="s">
         <v>63</v>
       </c>
-      <c r="C24" s="35" t="s">
+      <c r="C24" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="D24" s="36" t="s">
+      <c r="D24" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="E24" s="36">
+      <c r="E24" s="34">
         <v>8</v>
       </c>
-      <c r="F24" s="36">
+      <c r="F24" s="34">
         <v>6</v>
       </c>
-      <c r="G24" s="36" t="s">
+      <c r="G24" s="34" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="33" t="s">
+      <c r="A25" s="31" t="s">
         <v>64</v>
       </c>
-      <c r="B25" s="41" t="s">
+      <c r="B25" s="39" t="s">
         <v>65</v>
       </c>
-      <c r="C25" s="35" t="s">
+      <c r="C25" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="D25" s="36" t="s">
+      <c r="D25" s="34" t="s">
         <v>36</v>
       </c>
-      <c r="E25" s="36">
+      <c r="E25" s="34">
         <v>13</v>
       </c>
-      <c r="F25" s="36">
+      <c r="F25" s="34">
         <v>7</v>
       </c>
-      <c r="G25" s="36" t="s">
+      <c r="G25" s="34" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="42"/>
-      <c r="B26" s="43" t="s">
+      <c r="A26" s="40"/>
+      <c r="B26" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="C26" s="44"/>
-      <c r="D26" s="44"/>
-      <c r="E26" s="44"/>
-      <c r="F26" s="44"/>
-      <c r="G26" s="45"/>
+      <c r="C26" s="42"/>
+      <c r="D26" s="42"/>
+      <c r="E26" s="42"/>
+      <c r="F26" s="42"/>
+      <c r="G26" s="43"/>
     </row>
     <row r="27" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="46" t="s">
+      <c r="A27" s="44" t="s">
         <v>66</v>
       </c>
-      <c r="B27" s="47" t="s">
+      <c r="B27" s="45" t="s">
         <v>67</v>
       </c>
-      <c r="C27" s="48" t="s">
+      <c r="C27" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="D27" s="49" t="s">
+      <c r="D27" s="47" t="s">
         <v>36</v>
       </c>
-      <c r="E27" s="49">
+      <c r="E27" s="47">
         <v>13</v>
       </c>
-      <c r="F27" s="49">
+      <c r="F27" s="47">
         <v>4</v>
       </c>
-      <c r="G27" s="49" t="s">
+      <c r="G27" s="47" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="48" t="s">
         <v>68</v>
       </c>
-      <c r="B28" s="51" t="s">
+      <c r="B28" s="49" t="s">
         <v>69</v>
       </c>
-      <c r="C28" s="48" t="s">
+      <c r="C28" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="D28" s="49" t="s">
+      <c r="D28" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="E28" s="49">
+      <c r="E28" s="47">
         <v>8</v>
       </c>
-      <c r="F28" s="49">
+      <c r="F28" s="47">
         <v>5</v>
       </c>
-      <c r="G28" s="49" t="s">
+      <c r="G28" s="47" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="50" t="s">
+      <c r="A29" s="48" t="s">
         <v>70</v>
       </c>
-      <c r="B29" s="51" t="s">
+      <c r="B29" s="49" t="s">
         <v>71</v>
       </c>
-      <c r="C29" s="48" t="s">
+      <c r="C29" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="D29" s="49" t="s">
+      <c r="D29" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="E29" s="49">
+      <c r="E29" s="47">
         <v>8</v>
       </c>
-      <c r="F29" s="49">
+      <c r="F29" s="47">
         <v>6</v>
       </c>
-      <c r="G29" s="49" t="s">
+      <c r="G29" s="47" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="50" t="s">
+      <c r="A30" s="48" t="s">
         <v>72</v>
       </c>
-      <c r="B30" s="52" t="s">
+      <c r="B30" s="50" t="s">
         <v>73</v>
       </c>
-      <c r="C30" s="48" t="s">
+      <c r="C30" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="D30" s="49" t="s">
+      <c r="D30" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="E30" s="49">
+      <c r="E30" s="47">
         <v>8</v>
       </c>
-      <c r="F30" s="49">
+      <c r="F30" s="47">
         <v>8</v>
       </c>
-      <c r="G30" s="49" t="s">
+      <c r="G30" s="47" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="50" t="s">
+      <c r="A31" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="B31" s="52" t="s">
+      <c r="B31" s="50" t="s">
         <v>75</v>
       </c>
-      <c r="C31" s="48" t="s">
+      <c r="C31" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="D31" s="49" t="s">
+      <c r="D31" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="E31" s="49">
+      <c r="E31" s="47">
         <v>8</v>
       </c>
-      <c r="F31" s="49">
+      <c r="F31" s="47">
         <v>9</v>
       </c>
-      <c r="G31" s="49" t="s">
+      <c r="G31" s="47" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="50" t="s">
+      <c r="A32" s="48" t="s">
         <v>76</v>
       </c>
-      <c r="B32" s="52" t="s">
+      <c r="B32" s="50" t="s">
         <v>77</v>
       </c>
-      <c r="C32" s="48" t="s">
+      <c r="C32" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="D32" s="49" t="s">
+      <c r="D32" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="E32" s="49">
+      <c r="E32" s="47">
         <v>21</v>
       </c>
-      <c r="F32" s="49">
+      <c r="F32" s="47">
         <v>10</v>
       </c>
-      <c r="G32" s="49" t="s">
+      <c r="G32" s="47" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="50" t="s">
+      <c r="A33" s="48" t="s">
         <v>78</v>
       </c>
-      <c r="B33" s="52" t="s">
+      <c r="B33" s="50" t="s">
         <v>79</v>
       </c>
-      <c r="C33" s="48" t="s">
+      <c r="C33" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="D33" s="49" t="s">
+      <c r="D33" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="E33" s="49">
+      <c r="E33" s="47">
         <v>21</v>
       </c>
-      <c r="F33" s="49">
+      <c r="F33" s="47">
         <v>11</v>
       </c>
-      <c r="G33" s="49" t="s">
+      <c r="G33" s="47" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="46" t="s">
+      <c r="A34" s="44" t="s">
         <v>80</v>
       </c>
-      <c r="B34" s="51" t="s">
+      <c r="B34" s="49" t="s">
         <v>81</v>
       </c>
-      <c r="C34" s="48" t="s">
+      <c r="C34" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="D34" s="49" t="s">
+      <c r="D34" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="E34" s="49">
+      <c r="E34" s="47">
         <v>8</v>
       </c>
-      <c r="F34" s="49">
+      <c r="F34" s="47">
         <v>1</v>
       </c>
-      <c r="G34" s="49" t="s">
+      <c r="G34" s="47" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="46" t="s">
+      <c r="A35" s="44" t="s">
         <v>82</v>
       </c>
-      <c r="B35" s="51" t="s">
+      <c r="B35" s="49" t="s">
         <v>83</v>
       </c>
-      <c r="C35" s="48" t="s">
+      <c r="C35" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="D35" s="49" t="s">
+      <c r="D35" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="E35" s="49">
+      <c r="E35" s="47">
         <v>5</v>
       </c>
-      <c r="F35" s="49">
+      <c r="F35" s="47">
         <v>2</v>
       </c>
-      <c r="G35" s="49" t="s">
+      <c r="G35" s="47" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="46" t="s">
+      <c r="A36" s="44" t="s">
         <v>84</v>
       </c>
-      <c r="B36" s="51" t="s">
+      <c r="B36" s="49" t="s">
         <v>85</v>
       </c>
-      <c r="C36" s="48" t="s">
+      <c r="C36" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="D36" s="49" t="s">
+      <c r="D36" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="E36" s="49">
+      <c r="E36" s="47">
         <v>5</v>
       </c>
-      <c r="F36" s="49">
+      <c r="F36" s="47">
         <v>3</v>
       </c>
-      <c r="G36" s="49" t="s">
+      <c r="G36" s="47" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="50" t="s">
+      <c r="A37" s="48" t="s">
         <v>86</v>
       </c>
-      <c r="B37" s="51" t="s">
+      <c r="B37" s="49" t="s">
         <v>87</v>
       </c>
-      <c r="C37" s="48" t="s">
+      <c r="C37" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="D37" s="49" t="s">
+      <c r="D37" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="E37" s="49">
+      <c r="E37" s="47">
         <v>8</v>
       </c>
-      <c r="F37" s="49">
+      <c r="F37" s="47">
         <v>7</v>
       </c>
-      <c r="G37" s="49" t="s">
+      <c r="G37" s="47" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="50" t="s">
+      <c r="A38" s="48" t="s">
         <v>88</v>
       </c>
-      <c r="B38" s="53" t="s">
+      <c r="B38" s="51" t="s">
         <v>89</v>
       </c>
-      <c r="C38" s="48" t="s">
+      <c r="C38" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="D38" s="49" t="s">
+      <c r="D38" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="E38" s="49">
+      <c r="E38" s="47">
         <v>8</v>
       </c>
-      <c r="F38" s="49">
+      <c r="F38" s="47">
         <v>12</v>
       </c>
-      <c r="G38" s="49" t="s">
+      <c r="G38" s="47" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="54"/>
-      <c r="B39" s="55" t="s">
+      <c r="A39" s="52"/>
+      <c r="B39" s="53" t="s">
         <v>31</v>
       </c>
-      <c r="C39" s="56"/>
-      <c r="D39" s="56"/>
-      <c r="E39" s="56"/>
-      <c r="F39" s="56"/>
-      <c r="G39" s="57"/>
+      <c r="C39" s="54"/>
+      <c r="D39" s="54"/>
+      <c r="E39" s="54"/>
+      <c r="F39" s="54"/>
+      <c r="G39" s="55"/>
     </row>
     <row r="40" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="58" t="s">
+      <c r="A40" s="56" t="s">
         <v>90</v>
       </c>
-      <c r="B40" s="59" t="s">
+      <c r="B40" s="57" t="s">
         <v>91</v>
       </c>
-      <c r="C40" s="60" t="s">
+      <c r="C40" s="58" t="s">
         <v>92</v>
       </c>
-      <c r="D40" s="61" t="s">
+      <c r="D40" s="59" t="s">
         <v>18</v>
       </c>
-      <c r="E40" s="61">
+      <c r="E40" s="59">
         <v>5</v>
       </c>
-      <c r="F40" s="61">
+      <c r="F40" s="59">
         <v>3</v>
       </c>
-      <c r="G40" s="61" t="s">
+      <c r="G40" s="59" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="58" t="s">
+      <c r="A41" s="56" t="s">
         <v>93</v>
       </c>
-      <c r="B41" s="62" t="s">
+      <c r="B41" s="60" t="s">
         <v>94</v>
       </c>
-      <c r="C41" s="60" t="s">
+      <c r="C41" s="58" t="s">
         <v>92</v>
       </c>
-      <c r="D41" s="61" t="s">
+      <c r="D41" s="59" t="s">
         <v>18</v>
       </c>
-      <c r="E41" s="61">
+      <c r="E41" s="59">
         <v>5</v>
       </c>
-      <c r="F41" s="61">
+      <c r="F41" s="59">
         <v>4</v>
       </c>
-      <c r="G41" s="61" t="s">
+      <c r="G41" s="59" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="58" t="s">
+      <c r="A42" s="56" t="s">
         <v>95</v>
       </c>
-      <c r="B42" s="62" t="s">
+      <c r="B42" s="60" t="s">
         <v>96</v>
       </c>
-      <c r="C42" s="60" t="s">
+      <c r="C42" s="58" t="s">
         <v>92</v>
       </c>
-      <c r="D42" s="61" t="s">
+      <c r="D42" s="59" t="s">
         <v>39</v>
       </c>
-      <c r="E42" s="61">
+      <c r="E42" s="59">
         <v>3</v>
       </c>
-      <c r="F42" s="61">
+      <c r="F42" s="59">
         <v>1</v>
       </c>
-      <c r="G42" s="61" t="s">
+      <c r="G42" s="59" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="58" t="s">
+      <c r="A43" s="56" t="s">
         <v>97</v>
       </c>
-      <c r="B43" s="62" t="s">
+      <c r="B43" s="60" t="s">
         <v>98</v>
       </c>
-      <c r="C43" s="60" t="s">
+      <c r="C43" s="58" t="s">
         <v>92</v>
       </c>
-      <c r="D43" s="61" t="s">
+      <c r="D43" s="59" t="s">
         <v>39</v>
       </c>
-      <c r="E43" s="61">
+      <c r="E43" s="59">
         <v>3</v>
       </c>
-      <c r="F43" s="61">
+      <c r="F43" s="59">
         <v>2</v>
       </c>
-      <c r="G43" s="61" t="s">
+      <c r="G43" s="59" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="58" t="s">
+      <c r="A44" s="56" t="s">
         <v>99</v>
       </c>
-      <c r="B44" s="62" t="s">
+      <c r="B44" s="60" t="s">
         <v>100</v>
       </c>
-      <c r="C44" s="60" t="s">
+      <c r="C44" s="58" t="s">
         <v>92</v>
       </c>
-      <c r="D44" s="61" t="s">
+      <c r="D44" s="59" t="s">
         <v>27</v>
       </c>
-      <c r="E44" s="61">
+      <c r="E44" s="59">
         <v>21</v>
       </c>
-      <c r="F44" s="61">
+      <c r="F44" s="59">
         <v>5</v>
       </c>
-      <c r="G44" s="61" t="s">
+      <c r="G44" s="59" t="s">
         <v>31</v>
       </c>
     </row>
@@ -3678,258 +3691,283 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7428BDC3-EA57-423F-8C48-7A230F8D6310}">
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="7" width="18.5703125" customWidth="1"/>
+    <col min="2" max="2" width="50.5703125" customWidth="1"/>
+    <col min="3" max="8" width="18.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-    </row>
-    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="62"/>
+      <c r="G1" s="62"/>
+      <c r="H1" s="62"/>
+    </row>
+    <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>101</v>
       </c>
       <c r="B3" t="s">
+        <v>144</v>
+      </c>
+      <c r="C3" t="s">
         <v>102</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>103</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>104</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>105</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>106</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>145</v>
+      </c>
+      <c r="B4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>145</v>
+      </c>
+      <c r="B5" s="64"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="63" t="s">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="61" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="B21" s="61"/>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" s="63" t="s">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="61" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+      <c r="B32" s="61"/>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" s="63" t="s">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="61" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="B36" s="61"/>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>142</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
Continuando pt.1 -> 04.04.2026
</commit_message>
<xml_diff>
--- a/Backlog.xlsx
+++ b/Backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zdusa\OneDrive\Documentos\ZDU\Criacao de Jogos\Games\Clicker-Lizard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D12CBAA1-60A8-444F-949B-1A39A56053D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40DEF795-078F-4006-A505-89970F67BFAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,6 +19,9 @@
   <externalReferences>
     <externalReference r:id="rId3"/>
   </externalReferences>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Clicker Lizard'!$A$2:$J$41</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -40,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="163">
   <si>
     <t>PRODUCT BACKLOG - ZENLYX</t>
   </si>
@@ -605,27 +608,6 @@
     </r>
   </si>
   <si>
-    <t>Nome Requisito</t>
-  </si>
-  <si>
-    <t>Desc Requisito</t>
-  </si>
-  <si>
-    <t>Importante/Essencial/Desejavel</t>
-  </si>
-  <si>
-    <t>PP a GG</t>
-  </si>
-  <si>
-    <t>3 a 21</t>
-  </si>
-  <si>
-    <t>SLA</t>
-  </si>
-  <si>
-    <t>SPRINTS</t>
-  </si>
-  <si>
     <t>Click Padrão</t>
   </si>
   <si>
@@ -659,9 +641,6 @@
     <t>Sistema de Bloqueios</t>
   </si>
   <si>
-    <t>-----</t>
-  </si>
-  <si>
     <t>Vibração se possível</t>
   </si>
   <si>
@@ -734,19 +713,94 @@
     <t>Requisito Dividido</t>
   </si>
   <si>
-    <t>Parte do Requisito</t>
-  </si>
-  <si>
     <t>Layout</t>
   </si>
   <si>
     <t>Tela Inicial</t>
+  </si>
+  <si>
+    <t>Data Add</t>
+  </si>
+  <si>
+    <t>31/03/2026</t>
+  </si>
+  <si>
+    <t>Moeda Principal do Jogo</t>
+  </si>
+  <si>
+    <t>...</t>
+  </si>
+  <si>
+    <t>1 - Elemento Fogo...</t>
+  </si>
+  <si>
+    <t>Up 1- ...</t>
+  </si>
+  <si>
+    <t>Up Fogo 1- ...</t>
+  </si>
+  <si>
+    <t>Teste 1- ...</t>
+  </si>
+  <si>
+    <t>Pergunta 1- ...</t>
+  </si>
+  <si>
+    <t>Funcional / NF</t>
+  </si>
+  <si>
+    <t>Funcional</t>
+  </si>
+  <si>
+    <t>SPRINT 0</t>
+  </si>
+  <si>
+    <t>SPRINT 1</t>
+  </si>
+  <si>
+    <t>SPRINT 2</t>
+  </si>
+  <si>
+    <t>SPRINT 8</t>
+  </si>
+  <si>
+    <t>SPRINT 5</t>
+  </si>
+  <si>
+    <t>SPRINT 3</t>
+  </si>
+  <si>
+    <t>SPRINT 4</t>
+  </si>
+  <si>
+    <t>SPRINT 6</t>
+  </si>
+  <si>
+    <t>SPRINT 7</t>
+  </si>
+  <si>
+    <t>HTML/CSS da Tela Inicial</t>
+  </si>
+  <si>
+    <t>Sprint 5</t>
+  </si>
+  <si>
+    <t>Sprint 6</t>
+  </si>
+  <si>
+    <t>Sprint 7</t>
+  </si>
+  <si>
+    <t>Sprint 8</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd;@"/>
+  </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -982,7 +1036,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1121,7 +1175,49 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1636,6 +1732,504 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="pt-BR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="pt-BR"/>
+              <a:t>Gráfico de Burndown</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Clicker Lizard'!$O$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Estimativa da Sprint</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Clicker Lizard'!$L$3:$L$12</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>Total</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sprint 0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Sprint 1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Sprint 2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Sprint 3</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Sprint 4</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Sprint 5</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Sprint 6</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sprint 7</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Sprint 8</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Clicker Lizard'!$O$3:$O$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>425</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>360</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>295</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>248</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>212</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>175</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>131</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>84</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>63</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-10A4-4111-A13D-2C511CC08457}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Clicker Lizard'!$P$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Desempenho da Sprint</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Clicker Lizard'!$L$3:$L$12</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>Total</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sprint 0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Sprint 1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Sprint 2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Sprint 3</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Sprint 4</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Sprint 5</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Sprint 6</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sprint 7</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Sprint 8</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Clicker Lizard'!$P$3:$P$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>425</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>425</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>425</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>425</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>425</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>425</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>425</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>425</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>425</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>425</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-10A4-4111-A13D-2C511CC08457}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="177097920"/>
+        <c:axId val="177098880"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="177097920"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="pt-BR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="177098880"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="177098880"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="50000"/>
+                  <a:lumOff val="50000"/>
+                  <a:alpha val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="pt-BR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="177097920"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="50000"/>
+          <a:lumOff val="50000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="pt-BR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.511811024" r="0.511811024" t="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -1676,7 +2270,563 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2235,6 +3385,47 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>4762</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>4762</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>1042987</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>80962</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Gráfico 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AD027246-B300-198A-7E2C-2C8A17269DA2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
@@ -3691,15 +4882,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7428BDC3-EA57-423F-8C48-7A230F8D6310}">
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:P41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="50.5703125" customWidth="1"/>
-    <col min="3" max="8" width="18.5703125" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" customWidth="1"/>
+    <col min="3" max="3" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="9" width="15.140625" customWidth="1"/>
+    <col min="10" max="10" width="14.28515625" customWidth="1"/>
+    <col min="13" max="13" width="16" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="62" t="s">
         <v>0</v>
       </c>
@@ -3710,265 +4906,1344 @@
       <c r="F1" s="62"/>
       <c r="G1" s="62"/>
       <c r="H1" s="62"/>
-    </row>
-    <row r="2" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I1" s="62"/>
+      <c r="J1" s="62"/>
+      <c r="L1" s="63" t="s">
+        <v>1</v>
+      </c>
+      <c r="M1" s="63"/>
+      <c r="N1" s="63"/>
+      <c r="O1" s="63"/>
+      <c r="P1" s="63"/>
+    </row>
+    <row r="2" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="J2" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="L2" s="2"/>
+      <c r="M2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="66" t="s">
+        <v>136</v>
+      </c>
+      <c r="B3" s="66" t="s">
+        <v>137</v>
+      </c>
+      <c r="C3" s="67" t="s">
+        <v>158</v>
+      </c>
+      <c r="D3" s="67" t="s">
+        <v>148</v>
+      </c>
+      <c r="E3" s="67" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" s="67" t="s">
+        <v>36</v>
+      </c>
+      <c r="G3" s="67">
+        <v>13</v>
+      </c>
+      <c r="H3" s="67">
+        <v>1</v>
+      </c>
+      <c r="I3" s="67" t="s">
+        <v>149</v>
+      </c>
+      <c r="J3" s="68">
+        <v>46085</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="M3" s="9">
+        <f>SUM(G3:G37)</f>
+        <v>425</v>
+      </c>
+      <c r="N3" s="9">
+        <f>SUM(N4:N12)</f>
+        <v>0</v>
+      </c>
+      <c r="O3" s="9">
+        <f>M3</f>
+        <v>425</v>
+      </c>
+      <c r="P3" s="9">
+        <f>M3</f>
+        <v>425</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="66" t="s">
+        <v>125</v>
+      </c>
+      <c r="B4" s="69" t="s">
+        <v>141</v>
+      </c>
+      <c r="C4" s="67"/>
+      <c r="D4" s="67" t="s">
+        <v>148</v>
+      </c>
+      <c r="E4" s="67" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" s="67" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="67">
+        <v>21</v>
+      </c>
+      <c r="H4" s="67">
+        <v>1</v>
+      </c>
+      <c r="I4" s="67" t="s">
+        <v>149</v>
+      </c>
+      <c r="J4" s="68" t="s">
+        <v>139</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M4" s="9">
+        <f>SUM(G3:G7)</f>
+        <v>65</v>
+      </c>
+      <c r="N4" s="9">
+        <v>0</v>
+      </c>
+      <c r="O4" s="9">
+        <f t="shared" ref="O4:P6" si="0">O3-M4</f>
+        <v>360</v>
+      </c>
+      <c r="P4" s="9">
+        <f t="shared" si="0"/>
+        <v>425</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="66" t="s">
+        <v>126</v>
+      </c>
+      <c r="B5" s="66" t="s">
+        <v>141</v>
+      </c>
+      <c r="C5" s="67"/>
+      <c r="D5" s="67" t="s">
+        <v>148</v>
+      </c>
+      <c r="E5" s="67" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="67" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="67">
+        <v>5</v>
+      </c>
+      <c r="H5" s="67">
+        <v>1</v>
+      </c>
+      <c r="I5" s="67" t="s">
+        <v>149</v>
+      </c>
+      <c r="J5" s="68" t="s">
+        <v>139</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="M5" s="9">
+        <f>SUM(G8:G12)</f>
+        <v>65</v>
+      </c>
+      <c r="N5" s="9">
+        <v>0</v>
+      </c>
+      <c r="O5" s="9">
+        <f t="shared" si="0"/>
+        <v>295</v>
+      </c>
+      <c r="P5" s="9">
+        <f t="shared" si="0"/>
+        <v>425</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A6" s="66" t="s">
+        <v>127</v>
+      </c>
+      <c r="B6" s="66" t="s">
+        <v>141</v>
+      </c>
+      <c r="C6" s="67"/>
+      <c r="D6" s="67" t="s">
+        <v>148</v>
+      </c>
+      <c r="E6" s="67" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="67" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" s="67">
+        <v>13</v>
+      </c>
+      <c r="H6" s="67">
+        <v>2</v>
+      </c>
+      <c r="I6" s="67" t="s">
+        <v>149</v>
+      </c>
+      <c r="J6" s="68" t="s">
+        <v>139</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M6" s="9">
+        <f>SUM(G13:G15)</f>
+        <v>47</v>
+      </c>
+      <c r="N6" s="9">
+        <v>0</v>
+      </c>
+      <c r="O6" s="9">
+        <f t="shared" si="0"/>
+        <v>248</v>
+      </c>
+      <c r="P6" s="9">
+        <f t="shared" si="0"/>
+        <v>425</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" s="66" t="s">
+        <v>133</v>
+      </c>
+      <c r="B7" s="66" t="s">
+        <v>141</v>
+      </c>
+      <c r="C7" s="67"/>
+      <c r="D7" s="67" t="s">
+        <v>148</v>
+      </c>
+      <c r="E7" s="67" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" s="67" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" s="67">
+        <v>13</v>
+      </c>
+      <c r="H7" s="67">
+        <v>1</v>
+      </c>
+      <c r="I7" s="67" t="s">
+        <v>149</v>
+      </c>
+      <c r="J7" s="68" t="s">
+        <v>139</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M7" s="9">
+        <f>SUM(G16:G21)</f>
+        <v>36</v>
+      </c>
+      <c r="N7" s="9">
+        <v>0</v>
+      </c>
+      <c r="O7" s="9">
+        <f>O6-M7</f>
+        <v>212</v>
+      </c>
+      <c r="P7" s="9">
+        <f>P6-N7</f>
+        <v>425</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" s="70" t="s">
+        <v>102</v>
+      </c>
+      <c r="B8" s="70" t="s">
+        <v>141</v>
+      </c>
+      <c r="C8" s="71" t="s">
+        <v>140</v>
+      </c>
+      <c r="D8" s="71" t="s">
+        <v>148</v>
+      </c>
+      <c r="E8" s="71" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" s="71" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="71">
+        <v>5</v>
+      </c>
+      <c r="H8" s="71">
+        <v>1</v>
+      </c>
+      <c r="I8" s="71" t="s">
+        <v>150</v>
+      </c>
+      <c r="J8" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="M8" s="9">
+        <f>SUM(G22:G24)</f>
+        <v>37</v>
+      </c>
+      <c r="N8" s="9">
+        <v>0</v>
+      </c>
+      <c r="O8" s="9">
+        <f>O7-M8</f>
+        <v>175</v>
+      </c>
+      <c r="P8" s="9">
+        <f>P7-N8</f>
+        <v>425</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" s="70" t="s">
         <v>101</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B9" s="70" t="s">
+        <v>141</v>
+      </c>
+      <c r="C9" s="71"/>
+      <c r="D9" s="71" t="s">
+        <v>148</v>
+      </c>
+      <c r="E9" s="71" t="s">
+        <v>26</v>
+      </c>
+      <c r="F9" s="71" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" s="71">
+        <v>5</v>
+      </c>
+      <c r="H9" s="71">
+        <v>1</v>
+      </c>
+      <c r="I9" s="71" t="s">
+        <v>150</v>
+      </c>
+      <c r="J9" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="M9" s="9">
+        <f>SUM(G25:G29)</f>
+        <v>44</v>
+      </c>
+      <c r="N9" s="9">
+        <v>0</v>
+      </c>
+      <c r="O9" s="9">
+        <f t="shared" ref="O9:P11" si="1">O8-M9</f>
+        <v>131</v>
+      </c>
+      <c r="P9" s="9">
+        <f t="shared" si="1"/>
+        <v>425</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" s="70" t="s">
+        <v>103</v>
+      </c>
+      <c r="B10" s="70" t="s">
+        <v>141</v>
+      </c>
+      <c r="C10" s="71"/>
+      <c r="D10" s="71" t="s">
+        <v>148</v>
+      </c>
+      <c r="E10" s="71" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10" s="71" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" s="71">
+        <v>13</v>
+      </c>
+      <c r="H10" s="71">
+        <v>1</v>
+      </c>
+      <c r="I10" s="71" t="s">
+        <v>150</v>
+      </c>
+      <c r="J10" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="M10" s="9">
+        <f>SUM(G30:G33)</f>
+        <v>47</v>
+      </c>
+      <c r="N10" s="9">
+        <v>0</v>
+      </c>
+      <c r="O10" s="9">
+        <f t="shared" si="1"/>
+        <v>84</v>
+      </c>
+      <c r="P10" s="9">
+        <f t="shared" si="1"/>
+        <v>425</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" s="70" t="s">
+        <v>105</v>
+      </c>
+      <c r="B11" s="70" t="s">
+        <v>143</v>
+      </c>
+      <c r="C11" s="71"/>
+      <c r="D11" s="71" t="s">
+        <v>148</v>
+      </c>
+      <c r="E11" s="71" t="s">
+        <v>26</v>
+      </c>
+      <c r="F11" s="71" t="s">
+        <v>27</v>
+      </c>
+      <c r="G11" s="71">
+        <v>21</v>
+      </c>
+      <c r="H11" s="71">
+        <v>1</v>
+      </c>
+      <c r="I11" s="71" t="s">
+        <v>150</v>
+      </c>
+      <c r="J11" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="M11" s="9">
+        <f>SUM(G34)</f>
+        <v>21</v>
+      </c>
+      <c r="N11" s="9">
+        <v>0</v>
+      </c>
+      <c r="O11" s="9">
+        <f t="shared" si="1"/>
+        <v>63</v>
+      </c>
+      <c r="P11" s="9">
+        <f t="shared" si="1"/>
+        <v>425</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A12" s="70" t="s">
+        <v>128</v>
+      </c>
+      <c r="B12" s="70" t="s">
+        <v>141</v>
+      </c>
+      <c r="C12" s="71"/>
+      <c r="D12" s="71" t="s">
+        <v>148</v>
+      </c>
+      <c r="E12" s="71" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" s="71" t="s">
+        <v>27</v>
+      </c>
+      <c r="G12" s="71">
+        <v>21</v>
+      </c>
+      <c r="H12" s="71">
+        <v>1</v>
+      </c>
+      <c r="I12" s="71" t="s">
+        <v>150</v>
+      </c>
+      <c r="J12" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="M12" s="9">
+        <f>SUM(G35:G37)</f>
+        <v>63</v>
+      </c>
+      <c r="N12" s="9">
+        <v>0</v>
+      </c>
+      <c r="O12" s="9">
+        <f>O11-M12</f>
+        <v>0</v>
+      </c>
+      <c r="P12" s="9">
+        <f>P11-N12</f>
+        <v>425</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A13" s="73" t="s">
+        <v>104</v>
+      </c>
+      <c r="B13" s="73" t="s">
+        <v>142</v>
+      </c>
+      <c r="C13" s="74"/>
+      <c r="D13" s="74" t="s">
+        <v>148</v>
+      </c>
+      <c r="E13" s="74" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" s="74" t="s">
+        <v>27</v>
+      </c>
+      <c r="G13" s="74">
+        <v>21</v>
+      </c>
+      <c r="H13" s="74">
+        <v>1</v>
+      </c>
+      <c r="I13" s="74" t="s">
+        <v>151</v>
+      </c>
+      <c r="J13" s="75" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A14" s="73" t="s">
+        <v>106</v>
+      </c>
+      <c r="B14" s="73" t="s">
         <v>144</v>
       </c>
-      <c r="C3" t="s">
-        <v>102</v>
-      </c>
-      <c r="D3" t="s">
-        <v>103</v>
-      </c>
-      <c r="E3" t="s">
-        <v>104</v>
-      </c>
-      <c r="F3" t="s">
-        <v>105</v>
-      </c>
-      <c r="G3" t="s">
-        <v>106</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="C14" s="74"/>
+      <c r="D14" s="74" t="s">
+        <v>148</v>
+      </c>
+      <c r="E14" s="74" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" s="74" t="s">
+        <v>27</v>
+      </c>
+      <c r="G14" s="74">
+        <v>21</v>
+      </c>
+      <c r="H14" s="74">
+        <v>1</v>
+      </c>
+      <c r="I14" s="74" t="s">
+        <v>151</v>
+      </c>
+      <c r="J14" s="75" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A15" s="73" t="s">
+        <v>110</v>
+      </c>
+      <c r="B15" s="73" t="s">
+        <v>141</v>
+      </c>
+      <c r="C15" s="74"/>
+      <c r="D15" s="74" t="s">
+        <v>148</v>
+      </c>
+      <c r="E15" s="74" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" s="74" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" s="74">
+        <v>5</v>
+      </c>
+      <c r="H15" s="74">
+        <v>2</v>
+      </c>
+      <c r="I15" s="74" t="s">
+        <v>151</v>
+      </c>
+      <c r="J15" s="75" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A16" s="76" t="s">
+        <v>111</v>
+      </c>
+      <c r="B16" s="76" t="s">
+        <v>141</v>
+      </c>
+      <c r="C16" s="77"/>
+      <c r="D16" s="77" t="s">
+        <v>148</v>
+      </c>
+      <c r="E16" s="77" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" s="77" t="s">
+        <v>21</v>
+      </c>
+      <c r="G16" s="77">
+        <v>8</v>
+      </c>
+      <c r="H16" s="77">
+        <v>2</v>
+      </c>
+      <c r="I16" s="77" t="s">
+        <v>154</v>
+      </c>
+      <c r="J16" s="78" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="76" t="s">
+        <v>113</v>
+      </c>
+      <c r="B17" s="76" t="s">
+        <v>141</v>
+      </c>
+      <c r="C17" s="77"/>
+      <c r="D17" s="77" t="s">
+        <v>148</v>
+      </c>
+      <c r="E17" s="77" t="s">
+        <v>17</v>
+      </c>
+      <c r="F17" s="77" t="s">
+        <v>21</v>
+      </c>
+      <c r="G17" s="77">
+        <v>8</v>
+      </c>
+      <c r="H17" s="77">
+        <v>2</v>
+      </c>
+      <c r="I17" s="77" t="s">
+        <v>154</v>
+      </c>
+      <c r="J17" s="78" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="76" t="s">
+        <v>114</v>
+      </c>
+      <c r="B18" s="76" t="s">
+        <v>141</v>
+      </c>
+      <c r="C18" s="77"/>
+      <c r="D18" s="77" t="s">
+        <v>148</v>
+      </c>
+      <c r="E18" s="77" t="s">
+        <v>17</v>
+      </c>
+      <c r="F18" s="77" t="s">
+        <v>18</v>
+      </c>
+      <c r="G18" s="77">
+        <v>5</v>
+      </c>
+      <c r="H18" s="77">
+        <v>2</v>
+      </c>
+      <c r="I18" s="77" t="s">
+        <v>154</v>
+      </c>
+      <c r="J18" s="78" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="76" t="s">
+        <v>115</v>
+      </c>
+      <c r="B19" s="76" t="s">
+        <v>141</v>
+      </c>
+      <c r="C19" s="77"/>
+      <c r="D19" s="77" t="s">
+        <v>148</v>
+      </c>
+      <c r="E19" s="77" t="s">
+        <v>26</v>
+      </c>
+      <c r="F19" s="77" t="s">
+        <v>18</v>
+      </c>
+      <c r="G19" s="77">
+        <v>5</v>
+      </c>
+      <c r="H19" s="77">
+        <v>2</v>
+      </c>
+      <c r="I19" s="77" t="s">
+        <v>154</v>
+      </c>
+      <c r="J19" s="78" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="76" t="s">
+        <v>116</v>
+      </c>
+      <c r="B20" s="76" t="s">
+        <v>141</v>
+      </c>
+      <c r="C20" s="77"/>
+      <c r="D20" s="77" t="s">
+        <v>148</v>
+      </c>
+      <c r="E20" s="77" t="s">
+        <v>26</v>
+      </c>
+      <c r="F20" s="77" t="s">
+        <v>18</v>
+      </c>
+      <c r="G20" s="77">
+        <v>5</v>
+      </c>
+      <c r="H20" s="77">
+        <v>2</v>
+      </c>
+      <c r="I20" s="77" t="s">
+        <v>154</v>
+      </c>
+      <c r="J20" s="78" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="76" t="s">
+        <v>117</v>
+      </c>
+      <c r="B21" s="76" t="s">
+        <v>141</v>
+      </c>
+      <c r="C21" s="77"/>
+      <c r="D21" s="77" t="s">
+        <v>148</v>
+      </c>
+      <c r="E21" s="77" t="s">
+        <v>17</v>
+      </c>
+      <c r="F21" s="77" t="s">
+        <v>18</v>
+      </c>
+      <c r="G21" s="77">
+        <v>5</v>
+      </c>
+      <c r="H21" s="77">
+        <v>2</v>
+      </c>
+      <c r="I21" s="77" t="s">
+        <v>154</v>
+      </c>
+      <c r="J21" s="78" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" s="79" t="s">
+        <v>122</v>
+      </c>
+      <c r="B22" s="80" t="s">
+        <v>141</v>
+      </c>
+      <c r="C22" s="81"/>
+      <c r="D22" s="81" t="s">
+        <v>148</v>
+      </c>
+      <c r="E22" s="81" t="s">
+        <v>26</v>
+      </c>
+      <c r="F22" s="81" t="s">
+        <v>27</v>
+      </c>
+      <c r="G22" s="81">
+        <v>21</v>
+      </c>
+      <c r="H22" s="81">
+        <v>1</v>
+      </c>
+      <c r="I22" s="81" t="s">
+        <v>155</v>
+      </c>
+      <c r="J22" s="82" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="79" t="s">
+        <v>124</v>
+      </c>
+      <c r="B23" s="79" t="s">
+        <v>141</v>
+      </c>
+      <c r="C23" s="81"/>
+      <c r="D23" s="81" t="s">
+        <v>148</v>
+      </c>
+      <c r="E23" s="81" t="s">
+        <v>17</v>
+      </c>
+      <c r="F23" s="81" t="s">
+        <v>21</v>
+      </c>
+      <c r="G23" s="81">
+        <v>8</v>
+      </c>
+      <c r="H23" s="81">
+        <v>2</v>
+      </c>
+      <c r="I23" s="81" t="s">
+        <v>155</v>
+      </c>
+      <c r="J23" s="82" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="79" t="s">
+        <v>134</v>
+      </c>
+      <c r="B24" s="79" t="s">
+        <v>141</v>
+      </c>
+      <c r="C24" s="81"/>
+      <c r="D24" s="81" t="s">
+        <v>148</v>
+      </c>
+      <c r="E24" s="81" t="s">
+        <v>17</v>
+      </c>
+      <c r="F24" s="81" t="s">
+        <v>21</v>
+      </c>
+      <c r="G24" s="81">
+        <v>8</v>
+      </c>
+      <c r="H24" s="81">
+        <v>2</v>
+      </c>
+      <c r="I24" s="81" t="s">
+        <v>155</v>
+      </c>
+      <c r="J24" s="82" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>145</v>
-      </c>
-      <c r="B4" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>145</v>
-      </c>
-      <c r="B5" s="64"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="B25" t="s">
+        <v>141</v>
+      </c>
+      <c r="C25" s="64"/>
+      <c r="D25" s="64" t="s">
+        <v>148</v>
+      </c>
+      <c r="E25" s="64" t="s">
+        <v>17</v>
+      </c>
+      <c r="F25" s="64" t="s">
+        <v>21</v>
+      </c>
+      <c r="G25" s="64">
+        <v>8</v>
+      </c>
+      <c r="H25" s="64">
+        <v>3</v>
+      </c>
+      <c r="I25" s="64" t="s">
+        <v>153</v>
+      </c>
+      <c r="J25" s="65" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>123</v>
+      </c>
+      <c r="B26" t="s">
+        <v>141</v>
+      </c>
+      <c r="C26" s="64"/>
+      <c r="D26" s="64" t="s">
+        <v>148</v>
+      </c>
+      <c r="E26" s="64" t="s">
+        <v>26</v>
+      </c>
+      <c r="F26" s="64" t="s">
+        <v>36</v>
+      </c>
+      <c r="G26" s="64">
+        <v>13</v>
+      </c>
+      <c r="H26" s="64">
+        <v>2</v>
+      </c>
+      <c r="I26" s="64" t="s">
+        <v>153</v>
+      </c>
+      <c r="J26" s="65" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>108</v>
+      </c>
+      <c r="B27" t="s">
+        <v>141</v>
+      </c>
+      <c r="C27" s="64"/>
+      <c r="D27" s="64" t="s">
+        <v>148</v>
+      </c>
+      <c r="E27" s="64" t="s">
+        <v>17</v>
+      </c>
+      <c r="F27" s="64" t="s">
+        <v>18</v>
+      </c>
+      <c r="G27" s="64">
+        <v>5</v>
+      </c>
+      <c r="H27" s="64">
+        <v>3</v>
+      </c>
+      <c r="I27" s="64" t="s">
+        <v>153</v>
+      </c>
+      <c r="J27" s="65" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="B28" t="s">
+        <v>141</v>
+      </c>
+      <c r="C28" s="64"/>
+      <c r="D28" s="64" t="s">
+        <v>148</v>
+      </c>
+      <c r="E28" s="64" t="s">
+        <v>17</v>
+      </c>
+      <c r="F28" s="64" t="s">
+        <v>36</v>
+      </c>
+      <c r="G28" s="64">
+        <v>13</v>
+      </c>
+      <c r="H28" s="64">
+        <v>2</v>
+      </c>
+      <c r="I28" s="64" t="s">
+        <v>153</v>
+      </c>
+      <c r="J28" s="65" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="61" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>120</v>
-      </c>
-      <c r="B21" s="61"/>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B29" s="61" t="s">
+        <v>141</v>
+      </c>
+      <c r="C29" s="64"/>
+      <c r="D29" s="64" t="s">
+        <v>148</v>
+      </c>
+      <c r="E29" s="64" t="s">
+        <v>92</v>
+      </c>
+      <c r="F29" s="64" t="s">
+        <v>18</v>
+      </c>
+      <c r="G29" s="64">
+        <v>5</v>
+      </c>
+      <c r="H29" s="64">
+        <v>3</v>
+      </c>
+      <c r="I29" s="64" t="s">
+        <v>153</v>
+      </c>
+      <c r="J29" s="65" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="61" t="s">
+      <c r="B30" t="s">
+        <v>141</v>
+      </c>
+      <c r="C30" s="64"/>
+      <c r="D30" s="64" t="s">
+        <v>148</v>
+      </c>
+      <c r="E30" s="64" t="s">
+        <v>26</v>
+      </c>
+      <c r="F30" s="64" t="s">
+        <v>36</v>
+      </c>
+      <c r="G30" s="64">
+        <v>13</v>
+      </c>
+      <c r="H30" s="64">
+        <v>3</v>
+      </c>
+      <c r="I30" s="64" t="s">
+        <v>156</v>
+      </c>
+      <c r="J30" s="65" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>130</v>
+      </c>
+      <c r="B31" t="s">
+        <v>141</v>
+      </c>
+      <c r="C31" s="64"/>
+      <c r="D31" s="64" t="s">
+        <v>148</v>
+      </c>
+      <c r="E31" s="64" t="s">
+        <v>26</v>
+      </c>
+      <c r="F31" s="64" t="s">
+        <v>36</v>
+      </c>
+      <c r="G31" s="64">
+        <v>13</v>
+      </c>
+      <c r="H31" s="64">
+        <v>3</v>
+      </c>
+      <c r="I31" s="64" t="s">
+        <v>156</v>
+      </c>
+      <c r="J31" s="65" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>131</v>
+      </c>
+      <c r="B32" t="s">
+        <v>145</v>
+      </c>
+      <c r="C32" s="64"/>
+      <c r="D32" s="64" t="s">
+        <v>148</v>
+      </c>
+      <c r="E32" s="64" t="s">
+        <v>17</v>
+      </c>
+      <c r="F32" s="64" t="s">
+        <v>36</v>
+      </c>
+      <c r="G32" s="64">
+        <v>13</v>
+      </c>
+      <c r="H32" s="64">
+        <v>3</v>
+      </c>
+      <c r="I32" s="64" t="s">
+        <v>156</v>
+      </c>
+      <c r="J32" s="65" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>132</v>
+      </c>
+      <c r="B33" t="s">
+        <v>146</v>
+      </c>
+      <c r="C33" s="64"/>
+      <c r="D33" s="64" t="s">
+        <v>148</v>
+      </c>
+      <c r="E33" s="64" t="s">
+        <v>17</v>
+      </c>
+      <c r="F33" s="64" t="s">
+        <v>21</v>
+      </c>
+      <c r="G33" s="64">
+        <v>8</v>
+      </c>
+      <c r="H33" s="64">
+        <v>3</v>
+      </c>
+      <c r="I33" s="64" t="s">
+        <v>156</v>
+      </c>
+      <c r="J33" s="65" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>118</v>
+      </c>
+      <c r="B34" t="s">
+        <v>141</v>
+      </c>
+      <c r="C34" s="64"/>
+      <c r="D34" s="64" t="s">
+        <v>148</v>
+      </c>
+      <c r="E34" s="64" t="s">
+        <v>17</v>
+      </c>
+      <c r="F34" s="64" t="s">
+        <v>27</v>
+      </c>
+      <c r="G34" s="64">
+        <v>21</v>
+      </c>
+      <c r="H34" s="64">
+        <v>4</v>
+      </c>
+      <c r="I34" s="64" t="s">
+        <v>157</v>
+      </c>
+      <c r="J34" s="65" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>130</v>
-      </c>
-      <c r="B32" s="61"/>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="61" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B35" t="s">
+        <v>141</v>
+      </c>
+      <c r="C35" s="64"/>
+      <c r="D35" s="64" t="s">
+        <v>148</v>
+      </c>
+      <c r="E35" s="64" t="s">
+        <v>92</v>
+      </c>
+      <c r="F35" s="64" t="s">
+        <v>27</v>
+      </c>
+      <c r="G35" s="64">
+        <v>21</v>
+      </c>
+      <c r="H35" s="64">
+        <v>6</v>
+      </c>
+      <c r="I35" s="64" t="s">
+        <v>152</v>
+      </c>
+      <c r="J35" s="65" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>133</v>
-      </c>
-      <c r="B36" s="61"/>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+      <c r="B36" t="s">
+        <v>141</v>
+      </c>
+      <c r="C36" s="64"/>
+      <c r="D36" s="64" t="s">
+        <v>148</v>
+      </c>
+      <c r="E36" s="64" t="s">
+        <v>92</v>
+      </c>
+      <c r="F36" s="64" t="s">
+        <v>27</v>
+      </c>
+      <c r="G36" s="64">
+        <v>21</v>
+      </c>
+      <c r="H36" s="64">
+        <v>5</v>
+      </c>
+      <c r="I36" s="64" t="s">
+        <v>152</v>
+      </c>
+      <c r="J36" s="65" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+        <v>121</v>
+      </c>
+      <c r="B37" t="s">
+        <v>141</v>
+      </c>
+      <c r="C37" s="64"/>
+      <c r="D37" s="64" t="s">
+        <v>148</v>
+      </c>
+      <c r="E37" s="64" t="s">
+        <v>92</v>
+      </c>
+      <c r="F37" s="64" t="s">
+        <v>27</v>
+      </c>
+      <c r="G37" s="64">
+        <v>21</v>
+      </c>
+      <c r="H37" s="64">
+        <v>5</v>
+      </c>
+      <c r="I37" s="64" t="s">
+        <v>152</v>
+      </c>
+      <c r="J37" s="65" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>142</v>
-      </c>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C38" s="64"/>
+      <c r="D38" s="64"/>
+      <c r="E38" s="64"/>
+      <c r="F38" s="64"/>
+      <c r="G38" s="64"/>
+      <c r="H38" s="64"/>
+      <c r="I38" s="64"/>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" s="61"/>
+      <c r="C39" s="64"/>
+      <c r="D39" s="64"/>
+      <c r="E39" s="64"/>
+      <c r="F39" s="64"/>
+      <c r="G39" s="64"/>
+      <c r="H39" s="64"/>
+      <c r="I39" s="64"/>
+      <c r="J39" s="65"/>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A40" s="61"/>
+      <c r="C40" s="64"/>
+      <c r="D40" s="64"/>
+      <c r="E40" s="64"/>
+      <c r="F40" s="64"/>
+      <c r="G40" s="64"/>
+      <c r="H40" s="64"/>
+      <c r="I40" s="64"/>
+      <c r="J40" s="65"/>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A41" s="61"/>
+      <c r="C41" s="64"/>
+      <c r="D41" s="64"/>
+      <c r="E41" s="64"/>
+      <c r="F41" s="64"/>
+      <c r="G41" s="64"/>
+      <c r="H41" s="64"/>
+      <c r="I41" s="64"/>
+      <c r="J41" s="65"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="L1:P1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>